<commit_message>
Describe the margin method as a model limitation
"The model does not capture operating leverage because it forecasts profit as
a margin on revenue" in the Summary, Notes and README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tKeYTtjF85cuvm1dpYiVi
</commit_message>
<xml_diff>
--- a/model/GRG_model_v1.0.xlsx
+++ b/model/GRG_model_v1.0.xlsx
@@ -356,7 +356,7 @@
     <t xml:space="preserve">Key limitations</t>
   </si>
   <si>
-    <t xml:space="preserve">• Operating profit is a margin on revenue. Extra sales carry no operating leverage, and a sharp fall in sales would not squeeze the margin automatically, because fixed costs are not modelled separately.</t>
+    <t xml:space="preserve">• The model does not capture operating leverage because it forecasts operating profit as a margin on revenue; a sharp fall in sales would not squeeze the modelled margin automatically, because fixed costs are not modelled separately.</t>
   </si>
   <si>
     <t xml:space="preserve">• There is no separate impairment line, although recoverability of shop assets (IAS 36) is the auditor's key audit matter. FY22–FY25 margins absorbed £3–7m a year; a downside could bring larger charges than the margin allows for.</t>
@@ -521,7 +521,7 @@
     <t xml:space="preserve">5. Sensitivities: effect on underlying PBT (saved, base case)</t>
   </si>
   <si>
-    <t xml:space="preserve">Margin matters far more than sales growth: one point of margin moves FY26 profit by about £23m, one point of LFL by under £2m. Part of that is real (one point of LFL is about £19m of revenue, earning the 8.8% margin) and part is the margin method: extra sales carry no operating leverage, so in practice LFL would move profit more. The simulation partly allows for this by linking LFL and margin.</t>
+    <t xml:space="preserve">Margin matters far more than sales growth: one point of margin moves FY26 profit by about £23m, one point of LFL by under £2m. Part of that is real (one point of LFL is about £19m of revenue, earning the 8.8% margin) and part is the margin method: the model does not capture operating leverage because it forecasts profit as a margin on revenue, so in practice LFL would likely move profit more. The simulation partly allows for this by linking LFL and margin.</t>
   </si>
   <si>
     <t xml:space="preserve">6. Back-test: FY25 revenue method vs actual</t>
@@ -761,7 +761,7 @@
     <t xml:space="preserve">7.</t>
   </si>
   <si>
-    <t xml:space="preserve">Profit is a margin on revenue, so LFL growth carries no operating leverage outside the Monte Carlo (where LFL and margin are correlated at 0.5); each simulation run holds one draw per driver for all three years.</t>
+    <t xml:space="preserve">The model does not capture operating leverage because it forecasts profit as a margin on revenue (outside the Monte Carlo, where LFL and margin are correlated at 0.5); each simulation run holds one draw per driver for all three years.</t>
   </si>
   <si>
     <t xml:space="preserve">Data questions and how they were resolved</t>
@@ -3420,9 +3420,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>591480</xdr:colOff>
+      <xdr:colOff>591120</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>121320</xdr:rowOff>
+      <xdr:rowOff>120960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3436,7 +3436,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11466360" y="1036800"/>
-          <a:ext cx="6094800" cy="3199320"/>
+          <a:ext cx="6094440" cy="3198960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3457,9 +3457,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>591480</xdr:colOff>
+      <xdr:colOff>591120</xdr:colOff>
       <xdr:row>37</xdr:row>
-      <xdr:rowOff>6840</xdr:rowOff>
+      <xdr:rowOff>6480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3473,7 +3473,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="11466360" y="4656240"/>
-          <a:ext cx="6094800" cy="2894400"/>
+          <a:ext cx="6094440" cy="2894040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>